<commit_message>
Wrap table labels and record the ethnography proposal catalog
</commit_message>
<xml_diff>
--- a/review/museum-launch-map/museum-sequence.xlsx
+++ b/review/museum-launch-map/museum-sequence.xlsx
@@ -994,9 +994,8 @@
     </comment>
     <comment ref="J9" authorId="0" shapeId="0">
       <text>
-        <t>Три новых конкретных сценария для концепции, четыре развития и одно повторное использование. Строки ETN-N1–N8 внесены как идеи; код не начат. Время включено в исследование.
-Источник: Сергей, E-05; codex-bot, этап 2, 08.09.2026
-https://arabelthera-dot.github.io/rc-museum-preview/review/etnografiya/mechanisms.html</t>
+        <t>Изучены описания 85 базовых механик; отобраны 24 (16 предметных и 8 сопровождающих). Подготовлены предложения и 48 схематических состояний. Все 8 прежних сценариев по конкурентам остаются в реестре. Эти 24 предложения — предварительный задел: подбор под календарные дни и приёмка не выполнены этим каталогом.
+Источник: Собственный разбор и каталог Codex от 08.09.2026; текущий диалог с Сергеем.</t>
       </text>
     </comment>
     <comment ref="K9" authorId="0" shapeId="0">
@@ -7989,9 +7988,8 @@
     </comment>
     <comment ref="M9" authorId="0" shapeId="0">
       <text>
-        <t>Три новых конкретных сценария для концепции, четыре развития и одно повторное использование. Строки ETN-N1–N8 внесены как идеи; код не начат. Время включено в исследование.
-Источник: Сергей, E-05; codex-bot, этап 2, 08.09.2026
-https://arabelthera-dot.github.io/rc-museum-preview/review/etnografiya/mechanisms.html</t>
+        <t>Изучены описания 85 базовых механик; отобраны 24 (16 предметных и 8 сопровождающих). Подготовлены предложения и 48 схематических состояний. Все 8 прежних сценариев по конкурентам остаются в реестре. Эти 24 предложения — предварительный задел: подбор под календарные дни и приёмка не выполнены этим каталогом.
+Источник: Собственный разбор и каталог Codex от 08.09.2026; текущий диалог с Сергеем.</t>
       </text>
     </comment>
     <comment ref="N9" authorId="0" shapeId="0">
@@ -21160,7 +21158,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Порядок обновлён 08.09.2026 по поручению Сергея. Прежние фактические отметки сохранены; четыре новые проверки пока обозначены «?». Перенос граф не является новым аудитом готовности.</t>
+          <t>Порядок обновлён 08.09.2026 по поручению Сергея. Прежние отметки сохранены; уточнён только задел этнографии по завершённому в текущем диалоге каталогу: 24 предложения. Четыре новые проверки обозначены «?». Перенос граф не является новым аудитом готовности.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n"/>
@@ -22095,7 +22093,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>8 идей · ждут</t>
+          <t>24 предл.</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -28994,7 +28992,7 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>8 идей · ждут</t>
+          <t>24 предл.</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">

</xml_diff>